<commit_message>
update dataset prep final + some other updates
</commit_message>
<xml_diff>
--- a/data/input/mizuno.xlsx
+++ b/data/input/mizuno.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Saowalak/Desktop/CEOCommunication/data/preparation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Saowalak/Desktop/CEOCommunication/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{185B62C3-F115-404D-81F2-445CFD0FA989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D9F490-0814-504B-86C0-59AE282C8B98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="21560" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="153">
   <si>
     <t>ID</t>
   </si>
@@ -31,9 +31,6 @@
     <t>Text_type</t>
   </si>
   <si>
-    <t>new_name</t>
-  </si>
-  <si>
     <t>Information_valence_human</t>
   </si>
   <si>
@@ -85,9 +82,6 @@
     <t>neutral</t>
   </si>
   <si>
-    <t xml:space="preserve">message </t>
-  </si>
-  <si>
     <t>sustainability_report</t>
   </si>
   <si>
@@ -95,9 +89,6 @@
   </si>
   <si>
     <t>JPN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">president </t>
   </si>
   <si>
     <t>Akito Mizuno</t>
@@ -487,6 +478,9 @@
   </si>
   <si>
     <t>JPN25M06-00</t>
+  </si>
+  <si>
+    <t>Leadership_context_human</t>
   </si>
 </sst>
 </file>
@@ -539,6 +533,31 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9715E17C-372B-7542-BD8C-A03869F1D407}" name="Tableau1" displayName="Tableau1" ref="A1:P63" totalsRowShown="0">
+  <autoFilter ref="A1:P63" xr:uid="{9715E17C-372B-7542-BD8C-A03869F1D407}"/>
+  <tableColumns count="16">
+    <tableColumn id="1" xr3:uid="{41CF4C8B-3681-4F4F-9B9B-975B287E3290}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{75B0878A-B691-8644-90BF-9F2BACF8CE54}" name="Text"/>
+    <tableColumn id="3" xr3:uid="{1C9A8DC1-193D-464F-89AA-4617999451DA}" name="Text_type"/>
+    <tableColumn id="4" xr3:uid="{79619F63-261B-964D-BA57-87B16095E48F}" name="Leadership_context_human"/>
+    <tableColumn id="5" xr3:uid="{8D41BF09-2847-2947-B783-03C0AE4C56AA}" name="Information_valence_human"/>
+    <tableColumn id="6" xr3:uid="{DEDA7D19-19EE-F94D-9BDF-B365B07BE0D1}" name="Communication_type"/>
+    <tableColumn id="7" xr3:uid="{D89C5B20-7814-3F4A-8506-996FC55F4494}" name="Source_type "/>
+    <tableColumn id="8" xr3:uid="{42899E0D-FEFC-9F46-8088-E797A244E2BD}" name="Company"/>
+    <tableColumn id="9" xr3:uid="{2D2F3228-770A-A74F-8564-0024CAD6C943}" name="Country"/>
+    <tableColumn id="10" xr3:uid="{9C1C50DF-F6E1-B34F-80FB-CE72AF0F6D7B}" name="Year"/>
+    <tableColumn id="11" xr3:uid="{5A5D888E-50B5-3B46-BDE3-71FA5B120F36}" name="Covid"/>
+    <tableColumn id="12" xr3:uid="{BED9E0BB-5FC0-564D-B106-3ADB4FCD5E63}" name="Communicator_role"/>
+    <tableColumn id="13" xr3:uid="{88EC3125-87F9-974F-A600-EDAA24459933}" name="Communicator_name"/>
+    <tableColumn id="14" xr3:uid="{5E924055-0BB3-9043-9D26-58B877D4DF61}" name="Comment"/>
+    <tableColumn id="15" xr3:uid="{87DA28FD-121B-C34F-9FB4-AB7CA9DFCBE2}" name="Coding_ambiguity"/>
+    <tableColumn id="16" xr3:uid="{173CD1B6-5706-A34D-A599-7B5DD1E26B96}" name="Alternative_context"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -829,7 +848,18 @@
   <dimension ref="A1:P63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="25.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="34.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" customWidth="1"/>
+    <col min="9" max="9" width="9.6640625" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="15" max="15" width="17.33203125" customWidth="1"/>
+    <col min="16" max="16" width="18.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
@@ -843,72 +873,72 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
-      </c>
-      <c r="P1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>18</v>
       </c>
-      <c r="D2" t="s">
-        <v>19</v>
-      </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J2">
         <v>2021</v>
@@ -917,39 +947,39 @@
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
         <v>27</v>
       </c>
-      <c r="B3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" t="s">
-        <v>30</v>
-      </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J3">
         <v>2021</v>
@@ -958,39 +988,39 @@
         <v>1</v>
       </c>
       <c r="L3" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J4">
         <v>2021</v>
@@ -999,39 +1029,39 @@
         <v>1</v>
       </c>
       <c r="L4" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J5">
         <v>2021</v>
@@ -1040,39 +1070,39 @@
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J6">
         <v>2021</v>
@@ -1081,39 +1111,39 @@
         <v>1</v>
       </c>
       <c r="L6" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F7" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J7">
         <v>2021</v>
@@ -1122,39 +1152,39 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J8">
         <v>2021</v>
@@ -1163,39 +1193,39 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F9" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J9">
         <v>2021</v>
@@ -1204,39 +1234,39 @@
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F10" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J10">
         <v>2021</v>
@@ -1245,39 +1275,39 @@
         <v>1</v>
       </c>
       <c r="L10" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" t="s">
         <v>46</v>
       </c>
-      <c r="B11" t="s">
-        <v>47</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" t="s">
-        <v>49</v>
-      </c>
       <c r="F11" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J11">
         <v>2021</v>
@@ -1286,39 +1316,39 @@
         <v>1</v>
       </c>
       <c r="L11" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M11" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F12" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J12">
         <v>2022</v>
@@ -1327,39 +1357,39 @@
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="M12" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B13" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" t="s">
         <v>18</v>
       </c>
-      <c r="D13" t="s">
-        <v>19</v>
-      </c>
       <c r="E13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J13">
         <v>2022</v>
@@ -1368,39 +1398,39 @@
         <v>1</v>
       </c>
       <c r="L13" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M13" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B14" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F14" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J14">
         <v>2022</v>
@@ -1409,39 +1439,39 @@
         <v>1</v>
       </c>
       <c r="L14" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M14" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J15">
         <v>2022</v>
@@ -1450,39 +1480,39 @@
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M15" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C16" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D16" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G16" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I16" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J16">
         <v>2022</v>
@@ -1491,39 +1521,39 @@
         <v>1</v>
       </c>
       <c r="L16" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M16" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F17" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H17" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I17" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J17">
         <v>2022</v>
@@ -1532,39 +1562,39 @@
         <v>1</v>
       </c>
       <c r="L17" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M17" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C18" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D18" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F18" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J18">
         <v>2022</v>
@@ -1573,39 +1603,39 @@
         <v>1</v>
       </c>
       <c r="L18" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M18" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B19" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C19" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D19" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E19" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F19" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I19" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J19">
         <v>2022</v>
@@ -1614,39 +1644,39 @@
         <v>1</v>
       </c>
       <c r="L19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C20" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D20" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F20" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G20" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H20" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J20">
         <v>2022</v>
@@ -1655,39 +1685,39 @@
         <v>1</v>
       </c>
       <c r="L20" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M20" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B21" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D21" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F21" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H21" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J21">
         <v>2022</v>
@@ -1696,39 +1726,39 @@
         <v>1</v>
       </c>
       <c r="L21" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M21" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D22" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E22" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F22" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G22" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H22" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I22" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J22">
         <v>2023</v>
@@ -1737,39 +1767,39 @@
         <v>1</v>
       </c>
       <c r="L22" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M22" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C23" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D23" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G23" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I23" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J23">
         <v>2023</v>
@@ -1778,39 +1808,39 @@
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M23" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B24" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E24" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F24" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G24" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H24" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I24" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J24">
         <v>2023</v>
@@ -1819,39 +1849,39 @@
         <v>1</v>
       </c>
       <c r="L24" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M24" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C25" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D25" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E25" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F25" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G25" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H25" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I25" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J25">
         <v>2023</v>
@@ -1860,39 +1890,39 @@
         <v>1</v>
       </c>
       <c r="L25" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M25" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B26" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C26" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F26" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G26" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H26" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I26" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J26">
         <v>2023</v>
@@ -1901,39 +1931,39 @@
         <v>1</v>
       </c>
       <c r="L26" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M26" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B27" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C27" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D27" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F27" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H27" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I27" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J27">
         <v>2023</v>
@@ -1942,39 +1972,39 @@
         <v>1</v>
       </c>
       <c r="L27" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M27" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C28" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D28" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F28" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G28" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H28" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I28" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J28">
         <v>2023</v>
@@ -1983,39 +2013,39 @@
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M28" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C29" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D29" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E29" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F29" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G29" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H29" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I29" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J29">
         <v>2023</v>
@@ -2024,39 +2054,39 @@
         <v>1</v>
       </c>
       <c r="L29" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M29" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B30" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C30" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D30" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F30" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G30" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H30" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I30" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J30">
         <v>2023</v>
@@ -2065,39 +2095,39 @@
         <v>1</v>
       </c>
       <c r="L30" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M30" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C31" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" t="s">
         <v>18</v>
       </c>
-      <c r="D31" t="s">
-        <v>19</v>
-      </c>
       <c r="E31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F31" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G31" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H31" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I31" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J31">
         <v>2024</v>
@@ -2106,39 +2136,39 @@
         <v>0</v>
       </c>
       <c r="L31" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M31" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B32" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D32" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F32" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G32" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H32" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I32" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J32">
         <v>2024</v>
@@ -2147,39 +2177,39 @@
         <v>0</v>
       </c>
       <c r="L32" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M32" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C33" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D33" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E33" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F33" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G33" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H33" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I33" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J33">
         <v>2024</v>
@@ -2188,39 +2218,39 @@
         <v>0</v>
       </c>
       <c r="L33" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M33" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B34" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F34" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G34" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H34" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I34" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J34">
         <v>2024</v>
@@ -2229,39 +2259,39 @@
         <v>0</v>
       </c>
       <c r="L34" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M34" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B35" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C35" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D35" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E35" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F35" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G35" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H35" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I35" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J35">
         <v>2024</v>
@@ -2270,39 +2300,39 @@
         <v>0</v>
       </c>
       <c r="L35" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M35" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B36" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C36" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G36" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H36" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I36" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J36">
         <v>2024</v>
@@ -2311,39 +2341,39 @@
         <v>0</v>
       </c>
       <c r="L36" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M36" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B37" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D37" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E37" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F37" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G37" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H37" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I37" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J37">
         <v>2024</v>
@@ -2352,39 +2382,39 @@
         <v>0</v>
       </c>
       <c r="L37" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M37" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B38" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C38" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D38" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E38" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F38" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G38" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H38" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I38" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J38">
         <v>2024</v>
@@ -2393,39 +2423,39 @@
         <v>0</v>
       </c>
       <c r="L38" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M38" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B39" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C39" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D39" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E39" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F39" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G39" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H39" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I39" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J39">
         <v>2024</v>
@@ -2434,39 +2464,39 @@
         <v>0</v>
       </c>
       <c r="L39" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M39" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B40" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C40" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D40" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E40" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F40" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G40" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H40" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I40" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J40">
         <v>2024</v>
@@ -2475,39 +2505,39 @@
         <v>0</v>
       </c>
       <c r="L40" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M40" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B41" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D41" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E41" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F41" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G41" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H41" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I41" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J41">
         <v>2024</v>
@@ -2516,39 +2546,39 @@
         <v>0</v>
       </c>
       <c r="L41" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M41" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B42" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C42" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D42" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E42" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F42" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G42" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H42" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I42" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J42">
         <v>2024</v>
@@ -2557,39 +2587,39 @@
         <v>0</v>
       </c>
       <c r="L42" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M42" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B43" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C43" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D43" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E43" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F43" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G43" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H43" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I43" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J43">
         <v>2024</v>
@@ -2598,39 +2628,39 @@
         <v>0</v>
       </c>
       <c r="L43" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M43" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B44" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C44" t="s">
+        <v>17</v>
+      </c>
+      <c r="D44" t="s">
         <v>18</v>
       </c>
-      <c r="D44" t="s">
-        <v>19</v>
-      </c>
       <c r="E44" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F44" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G44" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H44" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I44" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J44">
         <v>2025</v>
@@ -2639,39 +2669,39 @@
         <v>0</v>
       </c>
       <c r="L44" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M44" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B45" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C45" t="s">
+        <v>17</v>
+      </c>
+      <c r="D45" t="s">
         <v>18</v>
       </c>
-      <c r="D45" t="s">
-        <v>19</v>
-      </c>
       <c r="E45" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F45" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G45" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H45" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I45" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J45">
         <v>2025</v>
@@ -2680,39 +2710,39 @@
         <v>0</v>
       </c>
       <c r="L45" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M45" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B46" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C46" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D46" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E46" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F46" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G46" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H46" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I46" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J46">
         <v>2025</v>
@@ -2721,39 +2751,39 @@
         <v>0</v>
       </c>
       <c r="L46" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M46" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B47" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C47" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D47" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E47" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F47" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G47" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H47" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I47" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J47">
         <v>2025</v>
@@ -2762,39 +2792,39 @@
         <v>0</v>
       </c>
       <c r="L47" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M47" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B48" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C48" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D48" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E48" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F48" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G48" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H48" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I48" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J48">
         <v>2025</v>
@@ -2803,39 +2833,39 @@
         <v>0</v>
       </c>
       <c r="L48" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M48" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B49" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C49" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D49" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E49" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F49" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G49" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H49" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I49" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J49">
         <v>2025</v>
@@ -2844,39 +2874,39 @@
         <v>0</v>
       </c>
       <c r="L49" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M49" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B50" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C50" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D50" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E50" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F50" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G50" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H50" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I50" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J50">
         <v>2025</v>
@@ -2885,39 +2915,39 @@
         <v>0</v>
       </c>
       <c r="L50" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M50" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B51" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C51" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D51" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E51" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F51" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G51" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H51" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I51" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J51">
         <v>2025</v>
@@ -2926,39 +2956,39 @@
         <v>0</v>
       </c>
       <c r="L51" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M51" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B52" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C52" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D52" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E52" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F52" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G52" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H52" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I52" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J52">
         <v>2025</v>
@@ -2967,39 +2997,39 @@
         <v>0</v>
       </c>
       <c r="L52" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M52" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B53" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C53" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D53" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E53" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F53" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G53" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H53" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I53" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J53">
         <v>2025</v>
@@ -3008,39 +3038,39 @@
         <v>0</v>
       </c>
       <c r="L53" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M53" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B54" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C54" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D54" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E54" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F54" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G54" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H54" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I54" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J54">
         <v>2025</v>
@@ -3049,39 +3079,39 @@
         <v>0</v>
       </c>
       <c r="L54" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M54" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B55" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C55" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D55" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E55" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F55" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G55" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H55" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I55" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J55">
         <v>2025</v>
@@ -3090,39 +3120,39 @@
         <v>0</v>
       </c>
       <c r="L55" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M55" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B56" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C56" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D56" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E56" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F56" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G56" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H56" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I56" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J56">
         <v>2025</v>
@@ -3131,39 +3161,39 @@
         <v>0</v>
       </c>
       <c r="L56" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M56" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B57" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C57" t="s">
+        <v>17</v>
+      </c>
+      <c r="D57" t="s">
         <v>18</v>
       </c>
-      <c r="D57" t="s">
-        <v>19</v>
-      </c>
       <c r="E57" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F57" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G57" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H57" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I57" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J57">
         <v>2025</v>
@@ -3172,39 +3202,39 @@
         <v>0</v>
       </c>
       <c r="L57" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M57" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B58" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C58" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D58" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E58" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F58" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G58" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H58" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I58" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J58">
         <v>2025</v>
@@ -3213,39 +3243,39 @@
         <v>0</v>
       </c>
       <c r="L58" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M58" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B59" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C59" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D59" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E59" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F59" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G59" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H59" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I59" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J59">
         <v>2025</v>
@@ -3254,39 +3284,39 @@
         <v>0</v>
       </c>
       <c r="L59" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M59" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B60" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C60" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D60" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E60" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F60" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G60" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H60" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I60" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J60">
         <v>2025</v>
@@ -3295,39 +3325,39 @@
         <v>0</v>
       </c>
       <c r="L60" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M60" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B61" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C61" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D61" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E61" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F61" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G61" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H61" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I61" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J61">
         <v>2025</v>
@@ -3336,39 +3366,39 @@
         <v>0</v>
       </c>
       <c r="L61" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M61" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B62" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C62" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D62" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E62" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F62" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G62" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H62" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I62" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J62">
         <v>2025</v>
@@ -3377,39 +3407,39 @@
         <v>0</v>
       </c>
       <c r="L62" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M62" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B63" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C63" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D63" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E63" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F63" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G63" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H63" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I63" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J63">
         <v>2025</v>
@@ -3418,13 +3448,16 @@
         <v>0</v>
       </c>
       <c r="L63" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M63" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>